<commit_message>
adjustes both queries and documents the evluation process
</commit_message>
<xml_diff>
--- a/RAG Evaluation manual.xlsx
+++ b/RAG Evaluation manual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A138A49-AD90-4542-819A-5EA2F15D968D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CE79AB-CB20-1348-8E3F-22BE5A1A5769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7700" yWindow="680" windowWidth="20940" windowHeight="16020" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
+    <workbookView xWindow="18240" yWindow="680" windowWidth="10420" windowHeight="16080" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t xml:space="preserve">Answer Relevancy
 Is the answer actually useful for the user’s query?
@@ -56,12 +56,6 @@
   </si>
   <si>
     <t>Query</t>
-  </si>
-  <si>
-    <t>How many jobs does the Great Barrier Reef generate in the whole of Australia?</t>
-  </si>
-  <si>
-    <t>How many jobs does the Great Barrier Reef generate locally?</t>
   </si>
   <si>
     <t xml:space="preserve">What is the value of the gross product which the Great Barrier Reef generates for Queensland? </t>
@@ -93,12 +87,6 @@
 destruction, less coral cover, less biodiversity (p. 5)</t>
   </si>
   <si>
-    <t>The Great Barrier Reef Marine Park (GBRMP) ranges from the tip of Cape York in
-Queensland in the north extending south past the Tropic of Capricorn almost to Bundaberg.
-It covers an area of approximately 345,400 square kilometres and stretches more than 2,300
-kilometres along the northeast coast of Queensland. (p. 11)</t>
-  </si>
-  <si>
     <t>How big is the Great Barrier Reef?</t>
   </si>
   <si>
@@ -132,13 +120,36 @@
     <t>Expected Text / Ground Truth</t>
   </si>
   <si>
-    <t>RAG Output</t>
-  </si>
-  <si>
     <t>Interpretation / Notes</t>
   </si>
   <si>
     <t>Evaluation metrics: relevant - partially relevant - not relevant</t>
+  </si>
+  <si>
+    <t>How many people work in the Great Barrier Reef industry in the whole of Australia?</t>
+  </si>
+  <si>
+    <t>How many persons in Queensland work at the Great Barrier Reef ?</t>
+  </si>
+  <si>
+    <t>How many people work locally at the Great Barrier Reef?</t>
+  </si>
+  <si>
+    <t>Whats the geografical range of the Great Barrier Reef?</t>
+  </si>
+  <si>
+    <t>It covers an area of approximately 345,400 square kilometres and stretches more than 2,300
+kilometres along the northeast coast of Queensland. (p. 11)</t>
+  </si>
+  <si>
+    <t>The Great Barrier Reef Marine Park (GBRMP) ranges from the tip of Cape York in
+Queensland in the north extending south past the Tropic of Capricorn almost to Bundaberg. (p.11)</t>
+  </si>
+  <si>
+    <t>RAG Output: Simple System-Prompt</t>
+  </si>
+  <si>
+    <t>RAG Output: Multiple Ruled System-Prompt</t>
   </si>
 </sst>
 </file>
@@ -525,151 +536,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{483B6C7E-3945-004D-9C20-B4D0D386A596}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="64.33203125" customWidth="1"/>
-    <col min="3" max="3" width="42.1640625" customWidth="1"/>
-    <col min="4" max="4" width="42.1640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="53.6640625" customWidth="1"/>
-    <col min="6" max="6" width="39.1640625" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="3" max="4" width="42.1640625" customWidth="1"/>
+    <col min="5" max="5" width="42.1640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="53.6640625" customWidth="1"/>
+    <col min="7" max="7" width="39.1640625" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="5"/>
-    </row>
-    <row r="6" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D6" s="5"/>
-    </row>
-    <row r="7" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="D7" s="5"/>
-    </row>
-    <row r="8" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D8" s="5"/>
-    </row>
-    <row r="9" spans="1:9" ht="170" x14ac:dyDescent="0.2">
+      <c r="E8" s="5"/>
+    </row>
+    <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D9" s="5"/>
-    </row>
-    <row r="10" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:10" ht="170" x14ac:dyDescent="0.2">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
implements two queries with same threshold and top_k to directly evaluate the system prompts; saves the example query in a cell.
</commit_message>
<xml_diff>
--- a/RAG Evaluation manual.xlsx
+++ b/RAG Evaluation manual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CE79AB-CB20-1348-8E3F-22BE5A1A5769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309C565C-E9A9-8641-8674-EFB123336D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18240" yWindow="680" windowWidth="10420" windowHeight="16080" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
+    <workbookView xWindow="5900" yWindow="680" windowWidth="22760" windowHeight="16080" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t xml:space="preserve">Answer Relevancy
 Is the answer actually useful for the user’s query?
@@ -129,9 +129,6 @@
     <t>How many people work in the Great Barrier Reef industry in the whole of Australia?</t>
   </si>
   <si>
-    <t>How many persons in Queensland work at the Great Barrier Reef ?</t>
-  </si>
-  <si>
     <t>How many people work locally at the Great Barrier Reef?</t>
   </si>
   <si>
@@ -150,6 +147,95 @@
   </si>
   <si>
     <t>RAG Output: Multiple Ruled System-Prompt</t>
+  </si>
+  <si>
+    <t>According to the provided context, the employment (full-time equivalent basis) for Australia is about 56,000 persons.</t>
+  </si>
+  <si>
+    <t>According to the provided context, approximately 56,000 persons are employed (on a full-time equivalent basis) in the Great Barrier Reef industry in Australia.</t>
+  </si>
+  <si>
+    <t>According to the context, approximately 44,000 persons work locally in the Great Barrier Reef region on a full-time equivalent basis.</t>
+  </si>
+  <si>
+    <t>According to the provided context, it is stated that "For employment (full time equivalent basis), about 66,000 persons." This refers to the total number of people employed in the tourism industry related to the Great Barrier Reef.</t>
+  </si>
+  <si>
+    <t>According to the provided context, about 56,000 persons (on a full-time equivalent basis) work in the Great Barrier Reef catchment area.</t>
+  </si>
+  <si>
+    <t>Answer: According to the provided context, it is mentioned that "For employment (full time equivalent basis), about 56,000 persons. The corresponding estimates for Australia are: For employment (full time equivalent basis), about 44,000 persons." Since we are looking at the number of persons working in Queensland, I will use the first estimate: about 56,000 persons. Answer: 56,000</t>
+  </si>
+  <si>
+    <t>How many persons in Queensland work at the Great Barrier Reef?</t>
+  </si>
+  <si>
+    <t>Around $5.4 billion per annum.</t>
+  </si>
+  <si>
+    <t>According to the provided context, the total economic contributions for Queensland (Table 7.2) show that the gross regional product for Queensland is around $5.4 billion per annum.
+Therefore, the answer is:
+$5.4 billion per annum</t>
+  </si>
+  <si>
+    <t>The symptoms of climate change at the Great Barrier Reef include:
+* Changes towards lower species diversity and numbers
+* Less coral cover
+* More specialisation on more hardy coral species
+* Higher algae concentrations</t>
+  </si>
+  <si>
+    <t>According to the provided context, the symptoms of climate change at the Great Barrier Reef (GBR) include:
+* Changes towards lower species diversity and numbers
+* Less coral cover
+* More specialisation on more hardy coral species
+* Higher algae concentrations
+These changes are attributed to atmospheric and cryospheric warming, ocean warming, sea level increases, and changes in ocean composition.</t>
+  </si>
+  <si>
+    <t>The geographical range of the Great Barrier Reef (GBRMP) is from the tip of Cape York in Queensland, extending south past the Tropic of Capricorn almost to Bundaberg, covering an area of approximately 345,400 square kilometres and stretching more than 2,300 kilometres along the northeast coast of Queensland.</t>
+  </si>
+  <si>
+    <t>The geographical range of the Great Barrier Reef (GBRMP) is from the tip of Cape York in Queensland, extending south past the Tropic of Capricorn almost to Bundaberg. It covers an area of approximately 345,400 square kilometres and stretches more than 2,300 kilometres along the northeast coast of Queensland.</t>
+  </si>
+  <si>
+    <t>The Great Barrier Reef covers an area of approximately 345,400 square kilometres and stretches over 2,300 kilometres along the northeast coast of Queensland.</t>
+  </si>
+  <si>
+    <t>According to the provided context, the width of the Park varies from around 90 kilometres to around 300 kilometres. However, this does not provide a direct answer to how big the Great Barrier Reef is in terms of area or total size.
+To find the area of the GBRMP, we can look at the text: "It covers an area of approximately 345,400 square kilometres..."</t>
+  </si>
+  <si>
+    <t>No, there is no recreational fishing licence fee for ocean fishing in Queensland.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I cannot find the answer. </t>
+  </si>
+  <si>
+    <t>The global average surface temperature has risen between 0.6 and 0.7 degrees Celsius since the start of the 20th century, and by 0.18 degrees Celsius per decade since then.</t>
+  </si>
+  <si>
+    <t>According to the provided context, it is stated that "Since the start of the 20th century, the global average surface temperature has risen between 0.6 and 0.7 degrees Celsius." Additionally, it is mentioned that "Since, the global average surface temperature has increased by 0.18 degrees Celsius per decade."
+To answer the question, I will calculate the total warming expected over a certain time period.
+Let's assume we want to know how much the Earth will warm up over the next century (from 2023 to 2123). To do this, we need to multiply the average annual increase in temperature by the number of years:
+0.18°C/decade × 10 decades = 1.8°C
+This means that the Earth is expected to warm up by approximately 1.8°C over the next century.
+Note: This calculation assumes a constant rate of warming, which may not be accurate due to various factors such as natural climate variability and potential changes in greenhouse gas emissions.</t>
+  </si>
+  <si>
+    <t>Atmospheric and cryospheric warming, changes in ocean composition (increased acidification), mass coral bleaching, increased extreme weather frequency, and disease vector movements are expected to directly affect tourism. These effects may lead to a decrease in the attractiveness of the Great Barrier Reef as a destination, as well as an increase in risks associated with visiting the area.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">According to the provided context, the climate change mechanisms directly affecting tourism are: * Atmospheric and cryospheric warming * Changes in ocean composition (increased acidification), which may lead to mass coral bleaching * Increased extreme weather frequency * Disease vector movements These effects will influence the attractiveness of the Great Barrier Reef as a destination, as well as the risks associated with visiting it. The impacts on tourism-related visitation and spending within the GBRCA are difficult to quantify due to broader economic drivers and substitution effects. In summary, climate change is expected to have negative impacts on tourism in the GBRCA, including reduced attractiveness, increased risks, and potential demand switch away from less cautiously-managed reef destinations. </t>
+  </si>
+  <si>
+    <t>The Great Barrier Reef gets approximately 2 million visits per year.</t>
+  </si>
+  <si>
+    <t>According to the context, Total reef visits increased from 1.4 million in-94 to just under 2 million visits in-05. However, there was a reduction of around 95,000 in-06.
+To find the average number of visits per year, we can calculate the average of these three values:
+(1,400,000 + 1,999,995 + 1,905,000) / 3 = 1,751,332.33
+So, on average, the Great Barrier Reef gets around 1.75 million visits per year.</t>
   </si>
 </sst>
 </file>
@@ -559,10 +645,10 @@
         <v>20</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -580,7 +666,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -590,33 +676,48 @@
       <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="136" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -626,9 +727,14 @@
       <c r="C5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+      <c r="D5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="221" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -638,23 +744,31 @@
       <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="D6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="119" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -662,10 +776,14 @@
         <v>12</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>26</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
@@ -677,10 +795,14 @@
       <c r="C9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="D9" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -690,10 +812,14 @@
       <c r="C10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" ht="170" x14ac:dyDescent="0.2">
+      <c r="D10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="306" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -703,10 +829,14 @@
       <c r="C11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="D11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="221" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -716,8 +846,12 @@
       <c r="C12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="D12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>